<commit_message>
#29 eSpark BOM updated
</commit_message>
<xml_diff>
--- a/Design Files/Baseboard-v2.0/BOM/eSpark_BOM_Baseboard-v2.0.xlsx
+++ b/Design Files/Baseboard-v2.0/BOM/eSpark_BOM_Baseboard-v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="821" uniqueCount="488">
   <si>
     <t>Component list</t>
   </si>
@@ -357,18 +357,9 @@
     <t>68uF 50V SMD,D6.3xL7.7mm Aluminum Electrolytic Capacitors - SMD ROHS</t>
   </si>
   <si>
-    <t>CAP ALUM 220UF 20% 50V SMD</t>
-  </si>
-  <si>
-    <t>CAP ALUM 10uF 25V SMD</t>
-  </si>
-  <si>
     <t>47uF 6.3V 5Ω@100kHz ±10% CASE-A-3216 Tantalum Capacitors ROHS</t>
   </si>
   <si>
-    <t>330uF 16V ±20% SMD,D6.3xL7.7mm Aluminum Electrolytic Capacitors - SMD ROHS</t>
-  </si>
-  <si>
     <t>CAP TANT 100UF 20% 10V 1411</t>
   </si>
   <si>
@@ -429,15 +420,9 @@
     <t>1x2P 18A -40℃~+105℃ 250V Black 12~30 Straight pin 5.08mm 2.5 1 2 Plugin,P=5.08mm Screw terminal ROHS</t>
   </si>
   <si>
-    <t>CONN HEADER SMD R/A 11POS 1.25MM</t>
-  </si>
-  <si>
     <t>1x6P SH 1 1mm 6 SMD,P=1mm Wire To Board / Wire To Wire Connector ROHS</t>
   </si>
   <si>
-    <t>CONN U.FL RCPT STR 50 OHM SMD</t>
-  </si>
-  <si>
     <t>0.8mm mPCI-E Surface Mount 52 SMD,P=0.8mm Card Edge Connectors ROHS</t>
   </si>
   <si>
@@ -597,9 +582,6 @@
     <t>Case-A</t>
   </si>
   <si>
-    <t>GVT1C331M0607</t>
-  </si>
-  <si>
     <t>Case-B</t>
   </si>
   <si>
@@ -639,12 +621,6 @@
     <t>DB128L-5.08-2P-BK-S</t>
   </si>
   <si>
-    <t>53261-1171</t>
-  </si>
-  <si>
-    <t>U.FL-R-SMT-1(80)</t>
-  </si>
-  <si>
     <t>91304-99-052R2</t>
   </si>
   <si>
@@ -741,12 +717,6 @@
     <t>CC0402KRX7R9BB103</t>
   </si>
   <si>
-    <t>UCD1H221MNL1GS</t>
-  </si>
-  <si>
-    <t>RVT1E100M0405</t>
-  </si>
-  <si>
     <t>CA45-A-6.3V-47uF-K</t>
   </si>
   <si>
@@ -936,15 +906,9 @@
     <t>ROQANG</t>
   </si>
   <si>
-    <t>Nichicon</t>
-  </si>
-  <si>
     <t>CEC</t>
   </si>
   <si>
-    <t>Honor Elec</t>
-  </si>
-  <si>
     <t>Kyocera AVX</t>
   </si>
   <si>
@@ -999,9 +963,6 @@
     <t>BOOMELE</t>
   </si>
   <si>
-    <t>Hirose</t>
-  </si>
-  <si>
     <t>UMAX</t>
   </si>
   <si>
@@ -1077,18 +1038,9 @@
     <t>C5221836</t>
   </si>
   <si>
-    <t>C116211</t>
-  </si>
-  <si>
-    <t>C970655</t>
-  </si>
-  <si>
     <t>C129570</t>
   </si>
   <si>
-    <t>C2980164</t>
-  </si>
-  <si>
     <t>C7196</t>
   </si>
   <si>
@@ -1143,9 +1095,6 @@
     <t>C430601</t>
   </si>
   <si>
-    <t>C585957</t>
-  </si>
-  <si>
     <t>C404126</t>
   </si>
   <si>
@@ -1428,9 +1377,6 @@
     <t>--</t>
   </si>
   <si>
-    <t>C88374</t>
-  </si>
-  <si>
     <t>C705793</t>
   </si>
   <si>
@@ -1482,7 +1428,61 @@
     <t>chipsmall</t>
   </si>
   <si>
-    <t>Quote Required</t>
+    <t>CONN HEADER SMD 11POS 1.25MM</t>
+  </si>
+  <si>
+    <t>53398-1171</t>
+  </si>
+  <si>
+    <t>1 Inner bore SMA Board Edge Bend -55℃~+155℃ 50Ω Plugin RF Connectors / Coaxial Connectors ROHS</t>
+  </si>
+  <si>
+    <t>HJ-SMA508</t>
+  </si>
+  <si>
+    <t>HJ Tech</t>
+  </si>
+  <si>
+    <t>C1509209</t>
+  </si>
+  <si>
+    <t>CAP TANT 220UF 10% 10V 2917</t>
+  </si>
+  <si>
+    <t>Case-D</t>
+  </si>
+  <si>
+    <t>TAJD227K010RNJV</t>
+  </si>
+  <si>
+    <t>C8024</t>
+  </si>
+  <si>
+    <t>10uF 10V 8Ω@100kHz ±10% CASE-A-3216 Tantalum Capacitors ROHS</t>
+  </si>
+  <si>
+    <t>CA45-A-10V-10uF-K</t>
+  </si>
+  <si>
+    <t>CEC(Shenzhen Zhenhua XinYun Elec)</t>
+  </si>
+  <si>
+    <t>C128253</t>
+  </si>
+  <si>
+    <t>CAP TANT 330UF 20% 16V 2917</t>
+  </si>
+  <si>
+    <t>Case-E</t>
+  </si>
+  <si>
+    <t>TAJE337M016RNJ</t>
+  </si>
+  <si>
+    <t>C51599</t>
+  </si>
+  <si>
+    <t>C504827</t>
   </si>
 </sst>
 </file>
@@ -2153,38 +2153,6 @@
     <xf numFmtId="0" fontId="23" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2219,6 +2187,38 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2596,15 +2596,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="68"/>
+      <c r="K1" s="80"/>
+      <c r="L1" s="80"/>
+      <c r="M1" s="80"/>
+      <c r="N1" s="80"/>
+      <c r="O1" s="80"/>
+      <c r="P1" s="80"/>
+      <c r="Q1" s="80"/>
+      <c r="R1" s="80"/>
+      <c r="S1" s="81"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="55" t="s">
-        <v>464</v>
+        <v>447</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="E3" s="13"/>
       <c r="F3" s="56" t="s">
-        <v>465</v>
+        <v>448</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="5"/>
@@ -2654,7 +2654,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="69"/>
+      <c r="S3" s="82"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2665,7 +2665,7 @@
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="57" t="s">
-        <v>465</v>
+        <v>448</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="7"/>
@@ -2679,7 +2679,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="70"/>
+      <c r="S4" s="83"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2704,7 +2704,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="70"/>
+      <c r="S5" s="83"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2725,7 +2725,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="70"/>
+      <c r="S6" s="83"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2746,7 +2746,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="70"/>
+      <c r="S7" s="83"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2767,7 +2767,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="70"/>
+      <c r="S8" s="83"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2784,46 +2784,46 @@
         <v>107</v>
       </c>
       <c r="F9" s="30" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="H9" s="30" t="s">
-        <v>301</v>
+        <v>291</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>451</v>
+        <v>434</v>
       </c>
       <c r="J9" s="30" t="s">
-        <v>347</v>
+        <v>334</v>
       </c>
       <c r="K9" s="30" t="s">
-        <v>459</v>
+        <v>442</v>
       </c>
       <c r="L9" s="30" t="s">
-        <v>450</v>
+        <v>433</v>
       </c>
       <c r="M9" s="30" t="s">
-        <v>458</v>
+        <v>441</v>
       </c>
       <c r="N9" s="30" t="s">
-        <v>452</v>
+        <v>435</v>
       </c>
       <c r="O9" s="30" t="s">
-        <v>453</v>
+        <v>436</v>
       </c>
       <c r="P9" s="30" t="s">
-        <v>454</v>
+        <v>437</v>
       </c>
       <c r="Q9" s="30" t="s">
-        <v>455</v>
+        <v>438</v>
       </c>
       <c r="R9" s="30" t="s">
-        <v>456</v>
+        <v>439</v>
       </c>
       <c r="S9" s="30" t="s">
-        <v>457</v>
+        <v>440</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
@@ -2833,31 +2833,31 @@
         <v>1</v>
       </c>
       <c r="C10" s="53" t="s">
-        <v>412</v>
+        <v>395</v>
       </c>
       <c r="D10" s="62" t="s">
         <v>28</v>
       </c>
       <c r="E10" s="62" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="F10" s="62" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="G10" s="62" t="s">
-        <v>412</v>
+        <v>395</v>
       </c>
       <c r="H10" s="66" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="I10" s="66" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J10" s="66" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="K10" s="62" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L10" s="62">
         <v>1</v>
@@ -2867,19 +2867,19 @@
         <v>5</v>
       </c>
       <c r="N10" s="62" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="O10" s="62" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="P10" s="66" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="Q10" s="66" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="R10" s="63" t="s">
-        <v>472</v>
+        <v>454</v>
       </c>
       <c r="S10" s="50"/>
     </row>
@@ -2899,22 +2899,22 @@
         <v>108</v>
       </c>
       <c r="F11" s="51" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="G11" s="51" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="H11" s="51" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I11" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J11" s="51" t="s">
-        <v>348</v>
+        <v>335</v>
       </c>
       <c r="K11" s="51" t="s">
-        <v>413</v>
+        <v>396</v>
       </c>
       <c r="L11" s="51">
         <v>1</v>
@@ -2927,7 +2927,7 @@
         <v>20</v>
       </c>
       <c r="O11" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P11" s="52">
         <v>2.01E-2</v>
@@ -2955,22 +2955,22 @@
         <v>109</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="G12" s="37" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="H12" s="37" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="I12" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J12" s="37" t="s">
-        <v>349</v>
+        <v>336</v>
       </c>
       <c r="K12" s="37" t="s">
-        <v>414</v>
+        <v>397</v>
       </c>
       <c r="L12" s="37">
         <v>25</v>
@@ -2983,7 +2983,7 @@
         <v>150</v>
       </c>
       <c r="O12" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P12" s="38">
         <v>1.0500000000000001E-2</v>
@@ -3011,22 +3011,22 @@
         <v>110</v>
       </c>
       <c r="F13" s="51" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="G13" s="51" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="H13" s="51" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I13" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J13" s="51" t="s">
-        <v>350</v>
+        <v>337</v>
       </c>
       <c r="K13" s="51" t="s">
-        <v>415</v>
+        <v>398</v>
       </c>
       <c r="L13" s="51">
         <v>3</v>
@@ -3039,7 +3039,7 @@
         <v>100</v>
       </c>
       <c r="O13" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P13" s="52">
         <v>8.9999999999999998E-4</v>
@@ -3067,22 +3067,22 @@
         <v>111</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G14" s="37" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="H14" s="37" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
       <c r="I14" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J14" s="37" t="s">
-        <v>351</v>
+        <v>338</v>
       </c>
       <c r="K14" s="37" t="s">
-        <v>416</v>
+        <v>399</v>
       </c>
       <c r="L14" s="37">
         <v>3</v>
@@ -3095,7 +3095,7 @@
         <v>20</v>
       </c>
       <c r="O14" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P14" s="38">
         <v>4.9099999999999998E-2</v>
@@ -3120,25 +3120,25 @@
         <v>33</v>
       </c>
       <c r="E15" s="51" t="s">
-        <v>112</v>
+        <v>475</v>
       </c>
       <c r="F15" s="51" t="s">
-        <v>466</v>
+        <v>476</v>
       </c>
       <c r="G15" s="51" t="s">
-        <v>240</v>
+        <v>477</v>
       </c>
       <c r="H15" s="51" t="s">
-        <v>305</v>
+        <v>296</v>
       </c>
       <c r="I15" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J15" s="51" t="s">
-        <v>352</v>
+        <v>478</v>
       </c>
       <c r="K15" s="51" t="s">
-        <v>417</v>
+        <v>400</v>
       </c>
       <c r="L15" s="51">
         <v>2</v>
@@ -3148,22 +3148,22 @@
         <v>10</v>
       </c>
       <c r="N15" s="51">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="O15" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P15" s="52">
-        <v>0.29670000000000002</v>
+        <v>0.27689999999999998</v>
       </c>
       <c r="Q15" s="52">
         <f t="shared" ref="Q15" si="6">P15*N15</f>
-        <v>4.4504999999999999</v>
+        <v>3.0458999999999996</v>
       </c>
       <c r="R15" s="51"/>
       <c r="S15" s="59"/>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="46">
         <f>ROW(B16) - ROW($B$9)</f>
@@ -3176,25 +3176,25 @@
         <v>34</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>113</v>
+        <v>479</v>
       </c>
       <c r="F16" s="37" t="s">
-        <v>466</v>
+        <v>186</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>241</v>
+        <v>480</v>
       </c>
       <c r="H16" s="37" t="s">
-        <v>304</v>
+        <v>481</v>
       </c>
       <c r="I16" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J16" s="37" t="s">
-        <v>353</v>
+        <v>482</v>
       </c>
       <c r="K16" s="37" t="s">
-        <v>418</v>
+        <v>401</v>
       </c>
       <c r="L16" s="37">
         <v>1</v>
@@ -3204,17 +3204,17 @@
         <v>5</v>
       </c>
       <c r="N16" s="37">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="O16" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P16" s="38">
-        <v>2.7099999999999999E-2</v>
+        <v>7.0900000000000005E-2</v>
       </c>
       <c r="Q16" s="38">
         <f>P16*N16</f>
-        <v>0.54200000000000004</v>
+        <v>1.0635000000000001</v>
       </c>
       <c r="R16" s="37"/>
       <c r="S16" s="59"/>
@@ -3232,25 +3232,25 @@
         <v>35</v>
       </c>
       <c r="E17" s="51" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F17" s="51" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="G17" s="51" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="H17" s="51" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="I17" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J17" s="51" t="s">
-        <v>354</v>
+        <v>339</v>
       </c>
       <c r="K17" s="51" t="s">
-        <v>419</v>
+        <v>402</v>
       </c>
       <c r="L17" s="51">
         <v>1</v>
@@ -3263,7 +3263,7 @@
         <v>10</v>
       </c>
       <c r="O17" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P17" s="52">
         <v>6.3E-2</v>
@@ -3275,7 +3275,7 @@
       <c r="R17" s="51"/>
       <c r="S17" s="59"/>
     </row>
-    <row r="18" spans="1:19" ht="36" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="46">
         <f>ROW(B18) - ROW($B$9)</f>
@@ -3288,25 +3288,25 @@
         <v>36</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>115</v>
+        <v>483</v>
       </c>
       <c r="F18" s="37" t="s">
-        <v>466</v>
+        <v>484</v>
       </c>
       <c r="G18" s="37" t="s">
-        <v>192</v>
+        <v>485</v>
       </c>
       <c r="H18" s="37" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="I18" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J18" s="37" t="s">
-        <v>355</v>
+        <v>486</v>
       </c>
       <c r="K18" s="37" t="s">
-        <v>420</v>
+        <v>403</v>
       </c>
       <c r="L18" s="37">
         <v>1</v>
@@ -3316,17 +3316,17 @@
         <v>5</v>
       </c>
       <c r="N18" s="37">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="O18" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P18" s="38">
-        <v>6.7199999999999996E-2</v>
+        <v>1.7373000000000001</v>
       </c>
       <c r="Q18" s="38">
         <f>P18*N18</f>
-        <v>0.67199999999999993</v>
+        <v>10.4238</v>
       </c>
       <c r="R18" s="37"/>
       <c r="S18" s="59"/>
@@ -3344,25 +3344,25 @@
         <v>37</v>
       </c>
       <c r="E19" s="51" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F19" s="51" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="G19" s="51" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="H19" s="51" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="I19" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J19" s="51" t="s">
-        <v>356</v>
+        <v>340</v>
       </c>
       <c r="K19" s="51" t="s">
-        <v>421</v>
+        <v>404</v>
       </c>
       <c r="L19" s="51">
         <v>1</v>
@@ -3375,7 +3375,7 @@
         <v>10</v>
       </c>
       <c r="O19" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P19" s="52">
         <v>0.26129999999999998</v>
@@ -3400,25 +3400,25 @@
         <v>38</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F20" s="37" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="G20" s="62" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="H20" s="37" t="s">
-        <v>309</v>
+        <v>297</v>
       </c>
       <c r="I20" s="37" t="s">
-        <v>474</v>
+        <v>456</v>
       </c>
       <c r="J20" s="37" t="s">
-        <v>473</v>
+        <v>455</v>
       </c>
       <c r="K20" s="37" t="s">
-        <v>422</v>
+        <v>405</v>
       </c>
       <c r="L20" s="37">
         <v>4</v>
@@ -3431,7 +3431,7 @@
         <v>30</v>
       </c>
       <c r="O20" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P20" s="38">
         <v>4.2000000000000003E-2</v>
@@ -3456,25 +3456,25 @@
         <v>39</v>
       </c>
       <c r="E21" s="51" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F21" s="51" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="G21" s="51" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="H21" s="51" t="s">
-        <v>310</v>
+        <v>298</v>
       </c>
       <c r="I21" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J21" s="51" t="s">
-        <v>357</v>
+        <v>341</v>
       </c>
       <c r="K21" s="51" t="s">
-        <v>418</v>
+        <v>401</v>
       </c>
       <c r="L21" s="51">
         <v>2</v>
@@ -3487,7 +3487,7 @@
         <v>50</v>
       </c>
       <c r="O21" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P21" s="52">
         <v>1.0800000000000001E-2</v>
@@ -3512,25 +3512,25 @@
         <v>40</v>
       </c>
       <c r="E22" s="37" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="F22" s="37" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="G22" s="37" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="H22" s="37" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I22" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J22" s="37" t="s">
-        <v>358</v>
+        <v>342</v>
       </c>
       <c r="K22" s="37" t="s">
-        <v>423</v>
+        <v>406</v>
       </c>
       <c r="L22" s="37">
         <v>2</v>
@@ -3543,7 +3543,7 @@
         <v>100</v>
       </c>
       <c r="O22" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P22" s="38">
         <v>1E-3</v>
@@ -3568,25 +3568,25 @@
         <v>41</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="F23" s="51" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="G23" s="51" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="H23" s="51" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I23" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J23" s="51" t="s">
-        <v>359</v>
+        <v>343</v>
       </c>
       <c r="K23" s="51" t="s">
-        <v>424</v>
+        <v>407</v>
       </c>
       <c r="L23" s="51">
         <v>3</v>
@@ -3599,7 +3599,7 @@
         <v>100</v>
       </c>
       <c r="O23" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P23" s="52">
         <v>3.8999999999999998E-3</v>
@@ -3624,25 +3624,25 @@
         <v>42</v>
       </c>
       <c r="E24" s="37" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F24" s="37" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="G24" s="37" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="H24" s="37" t="s">
-        <v>311</v>
+        <v>299</v>
       </c>
       <c r="I24" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J24" s="37" t="s">
-        <v>360</v>
+        <v>344</v>
       </c>
       <c r="K24" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L24" s="37">
         <v>1</v>
@@ -3655,7 +3655,7 @@
         <v>10</v>
       </c>
       <c r="O24" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P24" s="38">
         <v>5.5599999999999997E-2</v>
@@ -3680,25 +3680,25 @@
         <v>43</v>
       </c>
       <c r="E25" s="51" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F25" s="51" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="G25" s="51" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="H25" s="51" t="s">
-        <v>312</v>
+        <v>300</v>
       </c>
       <c r="I25" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J25" s="51" t="s">
-        <v>361</v>
+        <v>345</v>
       </c>
       <c r="K25" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L25" s="51">
         <v>1</v>
@@ -3711,7 +3711,7 @@
         <v>10</v>
       </c>
       <c r="O25" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P25" s="52">
         <v>4.4600000000000001E-2</v>
@@ -3736,25 +3736,25 @@
         <v>44</v>
       </c>
       <c r="E26" s="37" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="F26" s="37" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="G26" s="37" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="H26" s="37" t="s">
-        <v>313</v>
+        <v>301</v>
       </c>
       <c r="I26" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J26" s="37" t="s">
-        <v>362</v>
+        <v>346</v>
       </c>
       <c r="K26" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L26" s="37">
         <v>1</v>
@@ -3767,7 +3767,7 @@
         <v>6</v>
       </c>
       <c r="O26" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P26" s="38">
         <v>0.46939999999999998</v>
@@ -3792,25 +3792,25 @@
         <v>45</v>
       </c>
       <c r="E27" s="51" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="F27" s="51" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="G27" s="51" t="s">
-        <v>475</v>
+        <v>457</v>
       </c>
       <c r="H27" s="51" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="I27" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J27" s="51" t="s">
-        <v>476</v>
+        <v>458</v>
       </c>
       <c r="K27" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L27" s="51">
         <v>1</v>
@@ -3823,7 +3823,7 @@
         <v>10</v>
       </c>
       <c r="O27" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P27" s="52">
         <v>3.56E-2</v>
@@ -3848,25 +3848,25 @@
         <v>46</v>
       </c>
       <c r="E28" s="37" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F28" s="37" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="G28" s="37" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="H28" s="37" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
       <c r="I28" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J28" s="37" t="s">
-        <v>363</v>
+        <v>347</v>
       </c>
       <c r="K28" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L28" s="37">
         <v>3</v>
@@ -3879,7 +3879,7 @@
         <v>20</v>
       </c>
       <c r="O28" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P28" s="38">
         <v>2.46E-2</v>
@@ -3904,25 +3904,25 @@
         <v>47</v>
       </c>
       <c r="E29" s="51" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="F29" s="51" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="G29" s="51" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="H29" s="51" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="I29" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J29" s="51" t="s">
-        <v>364</v>
+        <v>348</v>
       </c>
       <c r="K29" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L29" s="51">
         <v>2</v>
@@ -3935,7 +3935,7 @@
         <v>20</v>
       </c>
       <c r="O29" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P29" s="52">
         <v>2.3400000000000001E-2</v>
@@ -3960,25 +3960,25 @@
         <v>48</v>
       </c>
       <c r="E30" s="37" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="F30" s="37" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="G30" s="37" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="H30" s="37" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="I30" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J30" s="37" t="s">
-        <v>365</v>
+        <v>349</v>
       </c>
       <c r="K30" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L30" s="37">
         <v>4</v>
@@ -3991,7 +3991,7 @@
         <v>25</v>
       </c>
       <c r="O30" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P30" s="38">
         <v>0.1351</v>
@@ -4016,25 +4016,25 @@
         <v>49</v>
       </c>
       <c r="E31" s="51" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F31" s="51" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="G31" s="51" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="H31" s="51" t="s">
-        <v>318</v>
+        <v>306</v>
       </c>
       <c r="I31" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J31" s="51" t="s">
-        <v>366</v>
+        <v>350</v>
       </c>
       <c r="K31" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L31" s="51">
         <v>4</v>
@@ -4047,7 +4047,7 @@
         <v>30</v>
       </c>
       <c r="O31" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P31" s="52">
         <v>4.7500000000000001E-2</v>
@@ -4072,25 +4072,25 @@
         <v>50</v>
       </c>
       <c r="E32" s="37" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="F32" s="37" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="G32" s="37" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="H32" s="37" t="s">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="I32" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J32" s="37" t="s">
-        <v>367</v>
+        <v>351</v>
       </c>
       <c r="K32" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L32" s="37">
         <v>1</v>
@@ -4103,7 +4103,7 @@
         <v>10</v>
       </c>
       <c r="O32" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P32" s="38">
         <v>0.2286</v>
@@ -4128,25 +4128,25 @@
         <v>51</v>
       </c>
       <c r="E33" s="51" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F33" s="51" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="G33" s="51" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="H33" s="51" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="I33" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J33" s="51" t="s">
-        <v>368</v>
+        <v>352</v>
       </c>
       <c r="K33" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L33" s="51">
         <v>1</v>
@@ -4159,7 +4159,7 @@
         <v>6</v>
       </c>
       <c r="O33" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P33" s="52">
         <v>1.1482000000000001</v>
@@ -4184,25 +4184,25 @@
         <v>52</v>
       </c>
       <c r="E34" s="37" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="F34" s="37" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="G34" s="37" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="H34" s="37" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="I34" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J34" s="37" t="s">
-        <v>369</v>
+        <v>353</v>
       </c>
       <c r="K34" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L34" s="37">
         <v>4</v>
@@ -4215,7 +4215,7 @@
         <v>30</v>
       </c>
       <c r="O34" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P34" s="38">
         <v>5.6099999999999997E-2</v>
@@ -4240,25 +4240,25 @@
         <v>53</v>
       </c>
       <c r="E35" s="51" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F35" s="51" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="G35" s="51" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="H35" s="51" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="I35" s="61" t="s">
-        <v>468</v>
+        <v>451</v>
       </c>
       <c r="J35" s="51" t="s">
-        <v>370</v>
+        <v>354</v>
       </c>
       <c r="K35" s="51" t="s">
-        <v>425</v>
+        <v>408</v>
       </c>
       <c r="L35" s="51">
         <v>1</v>
@@ -4271,7 +4271,7 @@
         <v>10</v>
       </c>
       <c r="O35" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P35" s="52">
         <v>8.8300000000000003E-2</v>
@@ -4296,25 +4296,25 @@
         <v>54</v>
       </c>
       <c r="E36" s="37" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="F36" s="51" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G36" s="37" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="H36" s="37" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
       <c r="I36" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J36" s="37" t="s">
-        <v>371</v>
+        <v>355</v>
       </c>
       <c r="K36" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L36" s="37">
         <v>8</v>
@@ -4327,7 +4327,7 @@
         <v>45</v>
       </c>
       <c r="O36" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P36" s="38">
         <v>0.2316</v>
@@ -4352,25 +4352,25 @@
         <v>55</v>
       </c>
       <c r="E37" s="51" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="F37" s="51" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G37" s="51" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="H37" s="51" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="I37" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J37" s="51" t="s">
-        <v>372</v>
+        <v>356</v>
       </c>
       <c r="K37" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L37" s="51">
         <v>1</v>
@@ -4383,7 +4383,7 @@
         <v>10</v>
       </c>
       <c r="O37" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P37" s="52">
         <v>0.21590000000000001</v>
@@ -4408,25 +4408,25 @@
         <v>56</v>
       </c>
       <c r="E38" s="37" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F38" s="51" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G38" s="37" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="H38" s="37" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
       <c r="I38" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J38" s="37" t="s">
-        <v>373</v>
+        <v>357</v>
       </c>
       <c r="K38" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L38" s="37">
         <v>4</v>
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="O38" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P38" s="38">
         <v>0.17299999999999999</v>
@@ -4464,25 +4464,25 @@
         <v>57</v>
       </c>
       <c r="E39" s="51" t="s">
-        <v>136</v>
+        <v>469</v>
       </c>
       <c r="F39" s="51" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G39" s="51" t="s">
-        <v>206</v>
+        <v>470</v>
       </c>
       <c r="H39" s="51" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="I39" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J39" s="51" t="s">
-        <v>374</v>
+        <v>487</v>
       </c>
       <c r="K39" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L39" s="51">
         <v>1</v>
@@ -4492,17 +4492,17 @@
         <v>5</v>
       </c>
       <c r="N39" s="51">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O39" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P39" s="52">
-        <v>0.36749999999999999</v>
+        <v>0.3211</v>
       </c>
       <c r="Q39" s="52">
         <f t="shared" ref="Q39" si="30">P39*N39</f>
-        <v>2.2050000000000001</v>
+        <v>3.2109999999999999</v>
       </c>
       <c r="R39" s="51"/>
       <c r="S39" s="59"/>
@@ -4520,25 +4520,25 @@
         <v>58</v>
       </c>
       <c r="E40" s="37" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="F40" s="51" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G40" s="37" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="H40" s="37" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="I40" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J40" s="37" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="K40" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L40" s="37">
         <v>1</v>
@@ -4551,7 +4551,7 @@
         <v>12</v>
       </c>
       <c r="O40" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P40" s="38">
         <v>7.0400000000000004E-2</v>
@@ -4563,38 +4563,36 @@
       <c r="R40" s="37"/>
       <c r="S40" s="59"/>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19" ht="36" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="47">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C41" s="54" t="s">
-        <v>461</v>
+        <v>444</v>
       </c>
       <c r="D41" s="51" t="s">
         <v>59</v>
       </c>
       <c r="E41" s="51" t="s">
-        <v>138</v>
+        <v>471</v>
       </c>
       <c r="F41" s="51" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G41" s="51" t="s">
-        <v>207</v>
+        <v>472</v>
       </c>
       <c r="H41" s="51" t="s">
-        <v>326</v>
-      </c>
-      <c r="I41" s="51" t="s">
-        <v>460</v>
-      </c>
+        <v>473</v>
+      </c>
+      <c r="I41" s="51"/>
       <c r="J41" s="51" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
       <c r="K41" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L41" s="51">
         <v>1</v>
@@ -4604,17 +4602,17 @@
         <v>5</v>
       </c>
       <c r="N41" s="51">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="O41" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P41" s="52">
-        <v>7.9600000000000004E-2</v>
+        <v>0.91159999999999997</v>
       </c>
       <c r="Q41" s="52">
         <f t="shared" ref="Q41" si="32">P41*N41</f>
-        <v>0.79600000000000004</v>
+        <v>5.4695999999999998</v>
       </c>
       <c r="R41" s="51"/>
       <c r="S41" s="59"/>
@@ -4632,25 +4630,25 @@
         <v>60</v>
       </c>
       <c r="E42" s="37" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="F42" s="51" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G42" s="37" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="H42" s="37" t="s">
-        <v>327</v>
+        <v>314</v>
       </c>
       <c r="I42" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J42" s="37" t="s">
-        <v>375</v>
+        <v>358</v>
       </c>
       <c r="K42" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L42" s="37">
         <v>2</v>
@@ -4663,7 +4661,7 @@
         <v>11</v>
       </c>
       <c r="O42" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P42" s="38">
         <v>0.81459999999999999</v>
@@ -4688,25 +4686,25 @@
         <v>61</v>
       </c>
       <c r="E43" s="51" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F43" s="51" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G43" s="51" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="H43" s="51" t="s">
-        <v>328</v>
+        <v>315</v>
       </c>
       <c r="I43" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J43" s="51" t="s">
-        <v>376</v>
+        <v>359</v>
       </c>
       <c r="K43" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L43" s="51">
         <v>3</v>
@@ -4719,7 +4717,7 @@
         <v>16</v>
       </c>
       <c r="O43" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P43" s="52">
         <v>0.32619999999999999</v>
@@ -4744,25 +4742,25 @@
         <v>62</v>
       </c>
       <c r="E44" s="37" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="F44" s="51" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G44" s="37" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="H44" s="37" t="s">
-        <v>329</v>
+        <v>316</v>
       </c>
       <c r="I44" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J44" s="37" t="s">
-        <v>377</v>
+        <v>360</v>
       </c>
       <c r="K44" s="37" t="s">
-        <v>426</v>
+        <v>409</v>
       </c>
       <c r="L44" s="37">
         <v>1</v>
@@ -4775,7 +4773,7 @@
         <v>10</v>
       </c>
       <c r="O44" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P44" s="38">
         <v>0.2137</v>
@@ -4800,25 +4798,25 @@
         <v>63</v>
       </c>
       <c r="E45" s="51" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="F45" s="51" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="G45" s="51" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="H45" s="51" t="s">
-        <v>330</v>
+        <v>317</v>
       </c>
       <c r="I45" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J45" s="51" t="s">
-        <v>378</v>
+        <v>361</v>
       </c>
       <c r="K45" s="51" t="s">
-        <v>427</v>
+        <v>410</v>
       </c>
       <c r="L45" s="51">
         <v>1</v>
@@ -4831,7 +4829,7 @@
         <v>50</v>
       </c>
       <c r="O45" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P45" s="52">
         <v>8.3000000000000001E-3</v>
@@ -4856,25 +4854,25 @@
         <v>64</v>
       </c>
       <c r="E46" s="37" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="F46" s="37" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="G46" s="37" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="H46" s="37" t="s">
-        <v>331</v>
+        <v>318</v>
       </c>
       <c r="I46" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J46" s="37" t="s">
-        <v>379</v>
+        <v>362</v>
       </c>
       <c r="K46" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L46" s="37">
         <v>2</v>
@@ -4887,7 +4885,7 @@
         <v>20</v>
       </c>
       <c r="O46" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P46" s="38">
         <v>5.7599999999999998E-2</v>
@@ -4912,25 +4910,25 @@
         <v>65</v>
       </c>
       <c r="E47" s="51" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="F47" s="51" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="G47" s="51" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="H47" s="51" t="s">
-        <v>331</v>
+        <v>318</v>
       </c>
       <c r="I47" s="61" t="s">
-        <v>468</v>
+        <v>451</v>
       </c>
       <c r="J47" s="51" t="s">
-        <v>380</v>
+        <v>363</v>
       </c>
       <c r="K47" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L47" s="51">
         <v>1</v>
@@ -4943,7 +4941,7 @@
         <v>10</v>
       </c>
       <c r="O47" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P47" s="52">
         <v>5.1499999999999997E-2</v>
@@ -4962,31 +4960,31 @@
         <v>39</v>
       </c>
       <c r="C48" s="53" t="s">
-        <v>462</v>
+        <v>445</v>
       </c>
       <c r="D48" s="62" t="s">
         <v>66</v>
       </c>
       <c r="E48" s="62" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="F48" s="62" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G48" s="62" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="H48" s="62" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="I48" s="62" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J48" s="62" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="K48" s="62" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L48" s="62">
         <v>10</v>
@@ -4996,19 +4994,19 @@
         <v>50</v>
       </c>
       <c r="N48" s="62" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="O48" s="62" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="P48" s="62" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="Q48" s="62" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="R48" s="63" t="s">
-        <v>472</v>
+        <v>454</v>
       </c>
       <c r="S48" s="59"/>
     </row>
@@ -5019,29 +5017,29 @@
         <v>40</v>
       </c>
       <c r="C49" s="54" t="s">
-        <v>463</v>
+        <v>446</v>
       </c>
       <c r="D49" s="51" t="s">
         <v>67</v>
       </c>
       <c r="E49" s="51" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="F49" s="51" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="G49" s="51" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="H49" s="51" t="s">
-        <v>332</v>
+        <v>319</v>
       </c>
       <c r="I49" s="51"/>
       <c r="J49" s="51" t="s">
-        <v>381</v>
+        <v>364</v>
       </c>
       <c r="K49" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L49" s="51">
         <v>1</v>
@@ -5054,7 +5052,7 @@
         <v>20</v>
       </c>
       <c r="O49" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P49" s="52">
         <v>2.1000000000000001E-2</v>
@@ -5079,25 +5077,25 @@
         <v>68</v>
       </c>
       <c r="E50" s="37" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="F50" s="37" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G50" s="62" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="H50" s="37" t="s">
-        <v>333</v>
+        <v>320</v>
       </c>
       <c r="I50" s="37" t="s">
-        <v>477</v>
+        <v>459</v>
       </c>
       <c r="J50" s="37" t="s">
-        <v>478</v>
+        <v>460</v>
       </c>
       <c r="K50" s="37" t="s">
-        <v>428</v>
+        <v>411</v>
       </c>
       <c r="L50" s="37">
         <v>2</v>
@@ -5110,7 +5108,7 @@
         <v>20</v>
       </c>
       <c r="O50" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P50" s="38">
         <v>2.1700000000000001E-2</v>
@@ -5135,23 +5133,23 @@
         <v>69</v>
       </c>
       <c r="E51" s="51" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="F51" s="51" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G51" s="51" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="H51" s="51" t="s">
-        <v>334</v>
+        <v>321</v>
       </c>
       <c r="I51" s="51"/>
       <c r="J51" s="51" t="s">
-        <v>382</v>
+        <v>365</v>
       </c>
       <c r="K51" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L51" s="51">
         <v>1</v>
@@ -5164,7 +5162,7 @@
         <v>10</v>
       </c>
       <c r="O51" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P51" s="52">
         <v>0.18260000000000001</v>
@@ -5189,23 +5187,23 @@
         <v>70</v>
       </c>
       <c r="E52" s="37" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="F52" s="37" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G52" s="37" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="H52" s="37" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I52" s="37"/>
       <c r="J52" s="37" t="s">
-        <v>383</v>
+        <v>366</v>
       </c>
       <c r="K52" s="37" t="s">
-        <v>429</v>
+        <v>412</v>
       </c>
       <c r="L52" s="37">
         <v>1</v>
@@ -5218,7 +5216,7 @@
         <v>100</v>
       </c>
       <c r="O52" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P52" s="38">
         <v>2.5999999999999999E-3</v>
@@ -5243,23 +5241,23 @@
         <v>71</v>
       </c>
       <c r="E53" s="51" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="F53" s="51" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="G53" s="51" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="H53" s="51" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I53" s="51"/>
       <c r="J53" s="51" t="s">
-        <v>384</v>
+        <v>367</v>
       </c>
       <c r="K53" s="51" t="s">
-        <v>430</v>
+        <v>413</v>
       </c>
       <c r="L53" s="51">
         <v>25</v>
@@ -5272,7 +5270,7 @@
         <v>200</v>
       </c>
       <c r="O53" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P53" s="52">
         <v>8.9999999999999998E-4</v>
@@ -5297,25 +5295,25 @@
         <v>72</v>
       </c>
       <c r="E54" s="37" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="F54" s="37" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="G54" s="62" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="H54" s="37" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I54" s="37" t="s">
-        <v>479</v>
+        <v>461</v>
       </c>
       <c r="J54" s="37" t="s">
-        <v>480</v>
+        <v>462</v>
       </c>
       <c r="K54" s="37" t="s">
-        <v>431</v>
+        <v>414</v>
       </c>
       <c r="L54" s="37">
         <v>7</v>
@@ -5328,7 +5326,7 @@
         <v>100</v>
       </c>
       <c r="O54" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P54" s="38">
         <v>8.9999999999999998E-4</v>
@@ -5353,25 +5351,25 @@
         <v>73</v>
       </c>
       <c r="E55" s="51" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="F55" s="51" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="G55" s="51" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="H55" s="51" t="s">
-        <v>335</v>
+        <v>322</v>
       </c>
       <c r="I55" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J55" s="51" t="s">
-        <v>385</v>
+        <v>368</v>
       </c>
       <c r="K55" s="51" t="s">
-        <v>432</v>
+        <v>415</v>
       </c>
       <c r="L55" s="51">
         <v>1</v>
@@ -5384,7 +5382,7 @@
         <v>100</v>
       </c>
       <c r="O55" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P55" s="52">
         <v>1E-3</v>
@@ -5409,25 +5407,25 @@
         <v>74</v>
       </c>
       <c r="E56" s="37" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="F56" s="37" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="G56" s="37" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="H56" s="37" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I56" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J56" s="37" t="s">
-        <v>386</v>
+        <v>369</v>
       </c>
       <c r="K56" s="37" t="s">
-        <v>433</v>
+        <v>416</v>
       </c>
       <c r="L56" s="37">
         <v>2</v>
@@ -5440,7 +5438,7 @@
         <v>100</v>
       </c>
       <c r="O56" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P56" s="38">
         <v>8.0000000000000004E-4</v>
@@ -5465,25 +5463,25 @@
         <v>75</v>
       </c>
       <c r="E57" s="51" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="F57" s="51" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="G57" s="62" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="H57" s="51" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I57" s="51" t="s">
-        <v>481</v>
+        <v>463</v>
       </c>
       <c r="J57" s="51" t="s">
-        <v>482</v>
+        <v>464</v>
       </c>
       <c r="K57" s="51" t="s">
-        <v>434</v>
+        <v>417</v>
       </c>
       <c r="L57" s="51">
         <v>1</v>
@@ -5496,7 +5494,7 @@
         <v>100</v>
       </c>
       <c r="O57" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P57" s="52">
         <v>5.0000000000000001E-4</v>
@@ -5521,23 +5519,23 @@
         <v>76</v>
       </c>
       <c r="E58" s="37" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="F58" s="37" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G58" s="37" t="s">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="H58" s="37" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I58" s="37"/>
       <c r="J58" s="37" t="s">
-        <v>387</v>
+        <v>370</v>
       </c>
       <c r="K58" s="37" t="s">
-        <v>435</v>
+        <v>418</v>
       </c>
       <c r="L58" s="37">
         <v>2</v>
@@ -5550,7 +5548,7 @@
         <v>100</v>
       </c>
       <c r="O58" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P58" s="38">
         <v>6.9999999999999999E-4</v>
@@ -5575,23 +5573,23 @@
         <v>77</v>
       </c>
       <c r="E59" s="51" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="F59" s="51" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G59" s="51" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="H59" s="51" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I59" s="51"/>
       <c r="J59" s="51" t="s">
-        <v>388</v>
+        <v>371</v>
       </c>
       <c r="K59" s="51" t="s">
-        <v>436</v>
+        <v>419</v>
       </c>
       <c r="L59" s="51">
         <v>22</v>
@@ -5604,7 +5602,7 @@
         <v>200</v>
       </c>
       <c r="O59" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P59" s="52">
         <v>6.9999999999999999E-4</v>
@@ -5629,23 +5627,23 @@
         <v>78</v>
       </c>
       <c r="E60" s="37" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="F60" s="37" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G60" s="37" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="H60" s="37" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I60" s="37"/>
       <c r="J60" s="37" t="s">
-        <v>389</v>
+        <v>372</v>
       </c>
       <c r="K60" s="37" t="s">
-        <v>437</v>
+        <v>420</v>
       </c>
       <c r="L60" s="37">
         <v>1</v>
@@ -5658,7 +5656,7 @@
         <v>100</v>
       </c>
       <c r="O60" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P60" s="38">
         <v>5.9999999999999995E-4</v>
@@ -5683,23 +5681,23 @@
         <v>79</v>
       </c>
       <c r="E61" s="37" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="F61" s="37" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G61" s="37" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="H61" s="37" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I61" s="37"/>
       <c r="J61" s="37" t="s">
-        <v>390</v>
+        <v>373</v>
       </c>
       <c r="K61" s="37" t="s">
-        <v>439</v>
+        <v>422</v>
       </c>
       <c r="L61" s="37">
         <v>4</v>
@@ -5712,7 +5710,7 @@
         <v>100</v>
       </c>
       <c r="O61" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P61" s="38">
         <v>6.9999999999999999E-4</v>
@@ -5737,23 +5735,23 @@
         <v>80</v>
       </c>
       <c r="E62" s="51" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F62" s="51" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="G62" s="51" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="H62" s="51" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I62" s="51"/>
       <c r="J62" s="51" t="s">
-        <v>391</v>
+        <v>374</v>
       </c>
       <c r="K62" s="51" t="s">
-        <v>440</v>
+        <v>423</v>
       </c>
       <c r="L62" s="51">
         <v>1</v>
@@ -5766,7 +5764,7 @@
         <v>100</v>
       </c>
       <c r="O62" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P62" s="52">
         <v>1.1999999999999999E-3</v>
@@ -5791,23 +5789,23 @@
         <v>81</v>
       </c>
       <c r="E63" s="37" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="F63" s="37" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G63" s="37" t="s">
-        <v>277</v>
+        <v>267</v>
       </c>
       <c r="H63" s="37" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I63" s="37"/>
       <c r="J63" s="37" t="s">
-        <v>392</v>
+        <v>375</v>
       </c>
       <c r="K63" s="37" t="s">
-        <v>441</v>
+        <v>424</v>
       </c>
       <c r="L63" s="37">
         <v>1</v>
@@ -5820,7 +5818,7 @@
         <v>100</v>
       </c>
       <c r="O63" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P63" s="38">
         <v>2.5000000000000001E-3</v>
@@ -5845,23 +5843,23 @@
         <v>82</v>
       </c>
       <c r="E64" s="51" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="F64" s="51" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="G64" s="51" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="H64" s="51" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I64" s="51"/>
       <c r="J64" s="51" t="s">
-        <v>470</v>
+        <v>452</v>
       </c>
       <c r="K64" s="51" t="s">
-        <v>442</v>
+        <v>425</v>
       </c>
       <c r="L64" s="51">
         <v>1</v>
@@ -5874,7 +5872,7 @@
         <v>20</v>
       </c>
       <c r="O64" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P64" s="52">
         <v>2.5999999999999999E-2</v>
@@ -5896,26 +5894,26 @@
         <v>21</v>
       </c>
       <c r="D65" s="51" t="s">
-        <v>485</v>
+        <v>467</v>
       </c>
       <c r="E65" s="37" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="F65" s="37" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G65" s="37" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
       <c r="H65" s="37" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I65" s="37"/>
       <c r="J65" s="37" t="s">
-        <v>393</v>
+        <v>376</v>
       </c>
       <c r="K65" s="37" t="s">
-        <v>438</v>
+        <v>421</v>
       </c>
       <c r="L65" s="37">
         <v>10</v>
@@ -5928,7 +5926,7 @@
         <v>100</v>
       </c>
       <c r="O65" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P65" s="38">
         <v>6.9999999999999999E-4</v>
@@ -5953,25 +5951,25 @@
         <v>83</v>
       </c>
       <c r="E66" s="51" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="F66" s="51" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G66" s="62" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="H66" s="51" t="s">
-        <v>336</v>
+        <v>323</v>
       </c>
       <c r="I66" s="51" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="J66" s="51" t="s">
-        <v>484</v>
+        <v>466</v>
       </c>
       <c r="K66" s="51" t="s">
-        <v>443</v>
+        <v>426</v>
       </c>
       <c r="L66" s="51">
         <v>4</v>
@@ -5984,7 +5982,7 @@
         <v>100</v>
       </c>
       <c r="O66" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P66" s="52">
         <v>4.0000000000000002E-4</v>
@@ -6009,23 +6007,23 @@
         <v>84</v>
       </c>
       <c r="E67" s="37" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="F67" s="37" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="G67" s="37" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="H67" s="37" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I67" s="37"/>
       <c r="J67" s="37" t="s">
-        <v>394</v>
+        <v>377</v>
       </c>
       <c r="K67" s="37" t="s">
-        <v>444</v>
+        <v>427</v>
       </c>
       <c r="L67" s="37">
         <v>1</v>
@@ -6038,7 +6036,7 @@
         <v>100</v>
       </c>
       <c r="O67" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P67" s="38">
         <v>1.1999999999999999E-3</v>
@@ -6063,23 +6061,23 @@
         <v>85</v>
       </c>
       <c r="E68" s="51" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="F68" s="51" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G68" s="51" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="H68" s="51" t="s">
-        <v>333</v>
+        <v>320</v>
       </c>
       <c r="I68" s="51"/>
       <c r="J68" s="51" t="s">
-        <v>395</v>
+        <v>378</v>
       </c>
       <c r="K68" s="51" t="s">
-        <v>445</v>
+        <v>428</v>
       </c>
       <c r="L68" s="51">
         <v>1</v>
@@ -6092,7 +6090,7 @@
         <v>10</v>
       </c>
       <c r="O68" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P68" s="52">
         <v>5.3600000000000002E-2</v>
@@ -6117,23 +6115,23 @@
         <v>86</v>
       </c>
       <c r="E69" s="37" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="F69" s="37" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="G69" s="37" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="H69" s="37" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I69" s="37"/>
       <c r="J69" s="37" t="s">
-        <v>396</v>
+        <v>379</v>
       </c>
       <c r="K69" s="37" t="s">
-        <v>446</v>
+        <v>429</v>
       </c>
       <c r="L69" s="37">
         <v>2</v>
@@ -6146,7 +6144,7 @@
         <v>100</v>
       </c>
       <c r="O69" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P69" s="38">
         <v>1.1999999999999999E-3</v>
@@ -6171,23 +6169,23 @@
         <v>87</v>
       </c>
       <c r="E70" s="51" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="F70" s="51" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G70" s="51" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="H70" s="51" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="I70" s="51"/>
       <c r="J70" s="51" t="s">
-        <v>397</v>
+        <v>380</v>
       </c>
       <c r="K70" s="51" t="s">
-        <v>447</v>
+        <v>430</v>
       </c>
       <c r="L70" s="51">
         <v>1</v>
@@ -6200,7 +6198,7 @@
         <v>100</v>
       </c>
       <c r="O70" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P70" s="52">
         <v>6.9999999999999999E-4</v>
@@ -6225,25 +6223,25 @@
         <v>88</v>
       </c>
       <c r="E71" s="64" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="F71" s="65" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G71" s="64" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="H71" s="64" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="I71" s="64" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J71" s="64" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="K71" s="64" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L71" s="64">
         <v>2</v>
@@ -6253,19 +6251,19 @@
         <v>10</v>
       </c>
       <c r="N71" s="64" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="O71" s="64" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="P71" s="64" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="Q71" s="64" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="R71" s="63" t="s">
-        <v>472</v>
+        <v>454</v>
       </c>
       <c r="S71" s="59"/>
     </row>
@@ -6282,25 +6280,25 @@
         <v>89</v>
       </c>
       <c r="E72" s="51" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="F72" s="51" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G72" s="51" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="H72" s="51" t="s">
-        <v>337</v>
+        <v>324</v>
       </c>
       <c r="I72" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J72" s="51" t="s">
-        <v>471</v>
+        <v>453</v>
       </c>
       <c r="K72" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L72" s="51">
         <v>1</v>
@@ -6313,7 +6311,7 @@
         <v>10</v>
       </c>
       <c r="O72" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P72" s="52">
         <v>0.1275</v>
@@ -6338,25 +6336,25 @@
         <v>90</v>
       </c>
       <c r="E73" s="37" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F73" s="37" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="G73" s="37" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="H73" s="37" t="s">
-        <v>338</v>
+        <v>325</v>
       </c>
       <c r="I73" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J73" s="37" t="s">
-        <v>398</v>
+        <v>381</v>
       </c>
       <c r="K73" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L73" s="37">
         <v>1</v>
@@ -6369,7 +6367,7 @@
         <v>6</v>
       </c>
       <c r="O73" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P73" s="38">
         <v>0.82569999999999999</v>
@@ -6394,25 +6392,25 @@
         <v>91</v>
       </c>
       <c r="E74" s="51" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="F74" s="51" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="G74" s="51" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="H74" s="51" t="s">
-        <v>338</v>
+        <v>325</v>
       </c>
       <c r="I74" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J74" s="51" t="s">
-        <v>399</v>
+        <v>382</v>
       </c>
       <c r="K74" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L74" s="51">
         <v>1</v>
@@ -6425,7 +6423,7 @@
         <v>6</v>
       </c>
       <c r="O74" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P74" s="52">
         <v>0.70009999999999994</v>
@@ -6450,25 +6448,25 @@
         <v>92</v>
       </c>
       <c r="E75" s="37" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="F75" s="37" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="G75" s="37" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="H75" s="37" t="s">
-        <v>339</v>
+        <v>326</v>
       </c>
       <c r="I75" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J75" s="37" t="s">
-        <v>400</v>
+        <v>383</v>
       </c>
       <c r="K75" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L75" s="37">
         <v>1</v>
@@ -6481,7 +6479,7 @@
         <v>10</v>
       </c>
       <c r="O75" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P75" s="38">
         <v>0.32279999999999998</v>
@@ -6506,25 +6504,25 @@
         <v>93</v>
       </c>
       <c r="E76" s="51" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="F76" s="51" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="G76" s="51" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="H76" s="51" t="s">
-        <v>340</v>
+        <v>327</v>
       </c>
       <c r="I76" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J76" s="51" t="s">
-        <v>401</v>
+        <v>384</v>
       </c>
       <c r="K76" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L76" s="51">
         <v>1</v>
@@ -6537,7 +6535,7 @@
         <v>6</v>
       </c>
       <c r="O76" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P76" s="52">
         <v>1.3062</v>
@@ -6562,23 +6560,23 @@
         <v>94</v>
       </c>
       <c r="E77" s="37" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="F77" s="37" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="G77" s="37" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="H77" s="37" t="s">
-        <v>341</v>
+        <v>328</v>
       </c>
       <c r="I77" s="37"/>
       <c r="J77" s="37" t="s">
-        <v>402</v>
+        <v>385</v>
       </c>
       <c r="K77" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L77" s="37">
         <v>1</v>
@@ -6591,7 +6589,7 @@
         <v>6</v>
       </c>
       <c r="O77" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P77" s="38">
         <v>0.3644</v>
@@ -6603,117 +6601,117 @@
       <c r="R77" s="37"/>
       <c r="S77" s="59"/>
     </row>
-    <row r="78" spans="1:19" s="84" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="77"/>
-      <c r="B78" s="78">
+    <row r="78" spans="1:19" s="74" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="67"/>
+      <c r="B78" s="68">
         <f t="shared" si="0"/>
         <v>69</v>
       </c>
-      <c r="C78" s="79" t="s">
+      <c r="C78" s="69" t="s">
         <v>25</v>
       </c>
-      <c r="D78" s="80" t="s">
+      <c r="D78" s="70" t="s">
         <v>95</v>
       </c>
-      <c r="E78" s="80" t="s">
-        <v>175</v>
-      </c>
-      <c r="F78" s="80" t="s">
-        <v>227</v>
-      </c>
-      <c r="G78" s="80" t="s">
-        <v>290</v>
-      </c>
-      <c r="H78" s="80" t="s">
-        <v>342</v>
-      </c>
-      <c r="I78" s="80" t="s">
-        <v>460</v>
-      </c>
-      <c r="J78" s="80" t="s">
-        <v>460</v>
-      </c>
-      <c r="K78" s="80" t="s">
-        <v>460</v>
-      </c>
-      <c r="L78" s="80">
+      <c r="E78" s="70" t="s">
+        <v>170</v>
+      </c>
+      <c r="F78" s="70" t="s">
+        <v>219</v>
+      </c>
+      <c r="G78" s="70" t="s">
+        <v>280</v>
+      </c>
+      <c r="H78" s="70" t="s">
+        <v>329</v>
+      </c>
+      <c r="I78" s="70" t="s">
+        <v>443</v>
+      </c>
+      <c r="J78" s="70" t="s">
+        <v>443</v>
+      </c>
+      <c r="K78" s="70" t="s">
+        <v>443</v>
+      </c>
+      <c r="L78" s="70">
         <v>1</v>
       </c>
-      <c r="M78" s="80">
+      <c r="M78" s="70">
         <f t="shared" ref="M78" si="67">L78*5</f>
         <v>5</v>
       </c>
-      <c r="N78" s="80">
+      <c r="N78" s="70">
         <v>6</v>
       </c>
-      <c r="O78" s="81" t="s">
-        <v>486</v>
-      </c>
-      <c r="P78" s="82">
+      <c r="O78" s="71" t="s">
+        <v>468</v>
+      </c>
+      <c r="P78" s="72">
         <v>2.5099999999999998</v>
       </c>
-      <c r="Q78" s="82">
+      <c r="Q78" s="72">
         <f t="shared" ref="Q78" si="68">P78*N78</f>
         <v>15.059999999999999</v>
       </c>
-      <c r="R78" s="80"/>
-      <c r="S78" s="83"/>
-    </row>
-    <row r="79" spans="1:19" s="84" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="77"/>
-      <c r="B79" s="85">
+      <c r="R78" s="70"/>
+      <c r="S78" s="73"/>
+    </row>
+    <row r="79" spans="1:19" s="74" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="67"/>
+      <c r="B79" s="75">
         <f>ROW(B79) - ROW($B$9)</f>
         <v>70</v>
       </c>
-      <c r="C79" s="86" t="s">
+      <c r="C79" s="76" t="s">
         <v>25</v>
       </c>
-      <c r="D79" s="87" t="s">
+      <c r="D79" s="77" t="s">
         <v>96</v>
       </c>
-      <c r="E79" s="87" t="s">
-        <v>176</v>
-      </c>
-      <c r="F79" s="87" t="s">
-        <v>228</v>
-      </c>
-      <c r="G79" s="87" t="s">
-        <v>291</v>
-      </c>
-      <c r="H79" s="87" t="s">
-        <v>340</v>
-      </c>
-      <c r="I79" s="87" t="s">
-        <v>460</v>
-      </c>
-      <c r="J79" s="87" t="s">
-        <v>460</v>
-      </c>
-      <c r="K79" s="87" t="s">
-        <v>460</v>
-      </c>
-      <c r="L79" s="87">
+      <c r="E79" s="77" t="s">
+        <v>171</v>
+      </c>
+      <c r="F79" s="77" t="s">
+        <v>220</v>
+      </c>
+      <c r="G79" s="77" t="s">
+        <v>281</v>
+      </c>
+      <c r="H79" s="77" t="s">
+        <v>327</v>
+      </c>
+      <c r="I79" s="77" t="s">
+        <v>443</v>
+      </c>
+      <c r="J79" s="77" t="s">
+        <v>443</v>
+      </c>
+      <c r="K79" s="77" t="s">
+        <v>443</v>
+      </c>
+      <c r="L79" s="77">
         <v>1</v>
       </c>
-      <c r="M79" s="87">
+      <c r="M79" s="77">
         <f>L79*5</f>
         <v>5</v>
       </c>
-      <c r="N79" s="87">
+      <c r="N79" s="77">
         <v>6</v>
       </c>
-      <c r="O79" s="81" t="s">
-        <v>486</v>
-      </c>
-      <c r="P79" s="88">
+      <c r="O79" s="71" t="s">
+        <v>468</v>
+      </c>
+      <c r="P79" s="78">
         <v>3.4329999999999998</v>
       </c>
-      <c r="Q79" s="88">
+      <c r="Q79" s="78">
         <f>P79*N79</f>
         <v>20.597999999999999</v>
       </c>
-      <c r="R79" s="87"/>
-      <c r="S79" s="83"/>
+      <c r="R79" s="77"/>
+      <c r="S79" s="73"/>
     </row>
     <row r="80" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A80" s="1"/>
@@ -6728,23 +6726,23 @@
         <v>97</v>
       </c>
       <c r="E80" s="51" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="F80" s="51" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="G80" s="51" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
       <c r="H80" s="51" t="s">
-        <v>343</v>
+        <v>330</v>
       </c>
       <c r="I80" s="51"/>
       <c r="J80" s="51" t="s">
-        <v>403</v>
+        <v>386</v>
       </c>
       <c r="K80" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L80" s="51">
         <v>1</v>
@@ -6757,7 +6755,7 @@
         <v>6</v>
       </c>
       <c r="O80" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P80" s="52">
         <v>4.6247999999999996</v>
@@ -6769,61 +6767,61 @@
       <c r="R80" s="51"/>
       <c r="S80" s="59"/>
     </row>
-    <row r="81" spans="1:19" s="84" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="77"/>
-      <c r="B81" s="85">
+    <row r="81" spans="1:19" s="74" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="67"/>
+      <c r="B81" s="75">
         <f>ROW(B81) - ROW($B$9)</f>
         <v>72</v>
       </c>
-      <c r="C81" s="86" t="s">
+      <c r="C81" s="76" t="s">
         <v>25</v>
       </c>
-      <c r="D81" s="87" t="s">
+      <c r="D81" s="77" t="s">
         <v>98</v>
       </c>
-      <c r="E81" s="87" t="s">
-        <v>178</v>
-      </c>
-      <c r="F81" s="87" t="s">
-        <v>230</v>
-      </c>
-      <c r="G81" s="87" t="s">
-        <v>293</v>
-      </c>
-      <c r="H81" s="87" t="s">
-        <v>344</v>
-      </c>
-      <c r="I81" s="87" t="s">
-        <v>460</v>
-      </c>
-      <c r="J81" s="87" t="s">
-        <v>460</v>
-      </c>
-      <c r="K81" s="87" t="s">
-        <v>460</v>
-      </c>
-      <c r="L81" s="87">
+      <c r="E81" s="77" t="s">
+        <v>173</v>
+      </c>
+      <c r="F81" s="77" t="s">
+        <v>222</v>
+      </c>
+      <c r="G81" s="77" t="s">
+        <v>283</v>
+      </c>
+      <c r="H81" s="77" t="s">
+        <v>331</v>
+      </c>
+      <c r="I81" s="77" t="s">
+        <v>443</v>
+      </c>
+      <c r="J81" s="77" t="s">
+        <v>443</v>
+      </c>
+      <c r="K81" s="77" t="s">
+        <v>443</v>
+      </c>
+      <c r="L81" s="77">
         <v>1</v>
       </c>
-      <c r="M81" s="87">
+      <c r="M81" s="77">
         <f>L81*5</f>
         <v>5</v>
       </c>
-      <c r="N81" s="87">
+      <c r="N81" s="77">
         <v>6</v>
       </c>
-      <c r="O81" s="81" t="s">
-        <v>486</v>
-      </c>
-      <c r="P81" s="88"/>
-      <c r="Q81" s="88">
+      <c r="O81" s="71" t="s">
+        <v>468</v>
+      </c>
+      <c r="P81" s="78">
+        <v>7.9</v>
+      </c>
+      <c r="Q81" s="78">
         <f>P81*N81</f>
-        <v>0</v>
-      </c>
-      <c r="R81" s="89" t="s">
-        <v>487</v>
-      </c>
-      <c r="S81" s="83"/>
+        <v>47.400000000000006</v>
+      </c>
+      <c r="R81" s="79"/>
+      <c r="S81" s="73"/>
     </row>
     <row r="82" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
@@ -6838,25 +6836,25 @@
         <v>99</v>
       </c>
       <c r="E82" s="51" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="F82" s="51" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="G82" s="51" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="H82" s="51" t="s">
-        <v>340</v>
+        <v>327</v>
       </c>
       <c r="I82" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J82" s="51" t="s">
-        <v>404</v>
+        <v>387</v>
       </c>
       <c r="K82" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L82" s="51">
         <v>3</v>
@@ -6869,7 +6867,7 @@
         <v>16</v>
       </c>
       <c r="O82" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P82" s="52">
         <v>1.7437</v>
@@ -6894,25 +6892,25 @@
         <v>100</v>
       </c>
       <c r="E83" s="37" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="F83" s="37" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="G83" s="37" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="H83" s="37" t="s">
-        <v>345</v>
+        <v>332</v>
       </c>
       <c r="I83" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J83" s="37" t="s">
-        <v>405</v>
+        <v>388</v>
       </c>
       <c r="K83" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L83" s="37">
         <v>1</v>
@@ -6925,7 +6923,7 @@
         <v>10</v>
       </c>
       <c r="O83" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P83" s="38">
         <v>7.7799999999999994E-2</v>
@@ -6950,25 +6948,25 @@
         <v>101</v>
       </c>
       <c r="E84" s="51" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="F84" s="51" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="G84" s="51" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="H84" s="51" t="s">
-        <v>338</v>
+        <v>325</v>
       </c>
       <c r="I84" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J84" s="51" t="s">
-        <v>406</v>
+        <v>389</v>
       </c>
       <c r="K84" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L84" s="51">
         <v>1</v>
@@ -6981,7 +6979,7 @@
         <v>6</v>
       </c>
       <c r="O84" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P84" s="52">
         <v>0.77800000000000002</v>
@@ -7006,25 +7004,25 @@
         <v>102</v>
       </c>
       <c r="E85" s="37" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="F85" s="37" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="G85" s="37" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
       <c r="H85" s="37" t="s">
-        <v>339</v>
+        <v>326</v>
       </c>
       <c r="I85" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J85" s="37" t="s">
-        <v>407</v>
+        <v>390</v>
       </c>
       <c r="K85" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L85" s="37">
         <v>1</v>
@@ -7037,7 +7035,7 @@
         <v>6</v>
       </c>
       <c r="O85" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P85" s="38">
         <v>0.41049999999999998</v>
@@ -7062,25 +7060,25 @@
         <v>103</v>
       </c>
       <c r="E86" s="51" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="F86" s="51" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="G86" s="51" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
       <c r="H86" s="51" t="s">
-        <v>344</v>
+        <v>331</v>
       </c>
       <c r="I86" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J86" s="51" t="s">
-        <v>408</v>
+        <v>391</v>
       </c>
       <c r="K86" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L86" s="51">
         <v>1</v>
@@ -7093,7 +7091,7 @@
         <v>6</v>
       </c>
       <c r="O86" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P86" s="52">
         <v>1.1837</v>
@@ -7118,25 +7116,25 @@
         <v>104</v>
       </c>
       <c r="E87" s="37" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="F87" s="37" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="G87" s="37" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
       <c r="H87" s="37" t="s">
-        <v>344</v>
+        <v>331</v>
       </c>
       <c r="I87" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J87" s="37" t="s">
-        <v>409</v>
+        <v>392</v>
       </c>
       <c r="K87" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="L87" s="37">
         <v>1</v>
@@ -7149,7 +7147,7 @@
         <v>6</v>
       </c>
       <c r="O87" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P87" s="38">
         <v>1.2107000000000001</v>
@@ -7174,25 +7172,25 @@
         <v>105</v>
       </c>
       <c r="E88" s="51" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="F88" s="51" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G88" s="51" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="H88" s="51" t="s">
-        <v>346</v>
+        <v>333</v>
       </c>
       <c r="I88" s="51" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J88" s="51" t="s">
-        <v>410</v>
+        <v>393</v>
       </c>
       <c r="K88" s="51" t="s">
-        <v>448</v>
+        <v>431</v>
       </c>
       <c r="L88" s="51">
         <v>1</v>
@@ -7205,7 +7203,7 @@
         <v>10</v>
       </c>
       <c r="O88" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P88" s="52">
         <v>0.08</v>
@@ -7230,25 +7228,25 @@
         <v>106</v>
       </c>
       <c r="E89" s="37" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="F89" s="51" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
       <c r="G89" s="37" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="H89" s="37" t="s">
-        <v>346</v>
+        <v>333</v>
       </c>
       <c r="I89" s="37" t="s">
-        <v>460</v>
+        <v>443</v>
       </c>
       <c r="J89" s="37" t="s">
-        <v>411</v>
+        <v>394</v>
       </c>
       <c r="K89" s="37" t="s">
-        <v>449</v>
+        <v>432</v>
       </c>
       <c r="L89" s="37">
         <v>1</v>
@@ -7261,7 +7259,7 @@
         <v>10</v>
       </c>
       <c r="O89" s="60" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
       <c r="P89" s="38">
         <v>8.0699999999999994E-2</v>
@@ -7287,17 +7285,17 @@
       <c r="K90" s="45"/>
       <c r="L90" s="45"/>
       <c r="M90" s="45"/>
-      <c r="N90" s="75" t="s">
+      <c r="N90" s="88" t="s">
         <v>5</v>
       </c>
-      <c r="O90" s="76"/>
-      <c r="P90" s="76"/>
+      <c r="O90" s="89"/>
+      <c r="P90" s="89"/>
       <c r="Q90" s="48">
         <f>SUM(Q10:Q89)</f>
-        <v>219.57099999999997</v>
-      </c>
-      <c r="R90" s="71"/>
-      <c r="S90" s="72"/>
+        <v>281.5193000000001</v>
+      </c>
+      <c r="R90" s="84"/>
+      <c r="S90" s="85"/>
     </row>
     <row r="91" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="1"/>
@@ -7313,17 +7311,17 @@
       <c r="K91" s="10"/>
       <c r="L91" s="10"/>
       <c r="M91" s="10"/>
-      <c r="N91" s="75" t="s">
+      <c r="N91" s="88" t="s">
         <v>6</v>
       </c>
-      <c r="O91" s="76"/>
-      <c r="P91" s="76"/>
+      <c r="O91" s="89"/>
+      <c r="P91" s="89"/>
       <c r="Q91" s="49">
         <f>Q90/5</f>
-        <v>43.914199999999994</v>
-      </c>
-      <c r="R91" s="73"/>
-      <c r="S91" s="74"/>
+        <v>56.303860000000022</v>
+      </c>
+      <c r="R91" s="86"/>
+      <c r="S91" s="87"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -7338,79 +7336,79 @@
     <hyperlink ref="O12" r:id="rId2"/>
     <hyperlink ref="O13" r:id="rId3"/>
     <hyperlink ref="O14" r:id="rId4"/>
-    <hyperlink ref="O15" r:id="rId5"/>
-    <hyperlink ref="O16" r:id="rId6"/>
-    <hyperlink ref="O17" r:id="rId7"/>
-    <hyperlink ref="O18" r:id="rId8"/>
-    <hyperlink ref="O19" r:id="rId9"/>
-    <hyperlink ref="O22" r:id="rId10"/>
-    <hyperlink ref="O21" r:id="rId11"/>
-    <hyperlink ref="O23" r:id="rId12"/>
-    <hyperlink ref="O24" r:id="rId13"/>
-    <hyperlink ref="O25" r:id="rId14"/>
-    <hyperlink ref="O28" r:id="rId15"/>
-    <hyperlink ref="O29" r:id="rId16"/>
-    <hyperlink ref="O30" r:id="rId17"/>
-    <hyperlink ref="O31" r:id="rId18"/>
-    <hyperlink ref="O32" r:id="rId19"/>
-    <hyperlink ref="O33" r:id="rId20"/>
-    <hyperlink ref="O34" r:id="rId21"/>
-    <hyperlink ref="O35" r:id="rId22"/>
-    <hyperlink ref="O36" r:id="rId23"/>
-    <hyperlink ref="O37" r:id="rId24"/>
-    <hyperlink ref="O38" r:id="rId25"/>
-    <hyperlink ref="O39" r:id="rId26"/>
-    <hyperlink ref="O40" r:id="rId27"/>
-    <hyperlink ref="O41" r:id="rId28"/>
-    <hyperlink ref="O42" r:id="rId29"/>
-    <hyperlink ref="O43" r:id="rId30"/>
-    <hyperlink ref="O44" r:id="rId31"/>
-    <hyperlink ref="O45" r:id="rId32"/>
-    <hyperlink ref="O46" r:id="rId33"/>
-    <hyperlink ref="O47" r:id="rId34"/>
-    <hyperlink ref="O49" r:id="rId35"/>
-    <hyperlink ref="O51" r:id="rId36"/>
-    <hyperlink ref="O52" r:id="rId37"/>
-    <hyperlink ref="O53" r:id="rId38"/>
-    <hyperlink ref="O55" r:id="rId39"/>
-    <hyperlink ref="O56" r:id="rId40"/>
-    <hyperlink ref="O58" r:id="rId41"/>
-    <hyperlink ref="O59" r:id="rId42"/>
-    <hyperlink ref="O60" r:id="rId43"/>
-    <hyperlink ref="O61" r:id="rId44"/>
-    <hyperlink ref="O62" r:id="rId45"/>
-    <hyperlink ref="O63" r:id="rId46"/>
-    <hyperlink ref="O64" r:id="rId47"/>
-    <hyperlink ref="O65" r:id="rId48"/>
-    <hyperlink ref="O67" r:id="rId49"/>
-    <hyperlink ref="O68" r:id="rId50"/>
-    <hyperlink ref="O69" r:id="rId51"/>
-    <hyperlink ref="O70" r:id="rId52"/>
-    <hyperlink ref="O73" r:id="rId53"/>
-    <hyperlink ref="O74" r:id="rId54"/>
-    <hyperlink ref="O75" r:id="rId55"/>
-    <hyperlink ref="O76" r:id="rId56"/>
-    <hyperlink ref="O77" r:id="rId57"/>
-    <hyperlink ref="O80" r:id="rId58"/>
-    <hyperlink ref="O82" r:id="rId59"/>
-    <hyperlink ref="O83" r:id="rId60"/>
-    <hyperlink ref="O84" r:id="rId61"/>
-    <hyperlink ref="O85" r:id="rId62"/>
-    <hyperlink ref="O86" r:id="rId63"/>
-    <hyperlink ref="O87" r:id="rId64"/>
-    <hyperlink ref="O88" r:id="rId65"/>
-    <hyperlink ref="O89" r:id="rId66"/>
-    <hyperlink ref="O72" r:id="rId67"/>
-    <hyperlink ref="O20" r:id="rId68"/>
-    <hyperlink ref="O26" r:id="rId69"/>
-    <hyperlink ref="O27" r:id="rId70"/>
-    <hyperlink ref="O50" r:id="rId71"/>
-    <hyperlink ref="O54" r:id="rId72"/>
-    <hyperlink ref="O57" r:id="rId73"/>
-    <hyperlink ref="O66" r:id="rId74"/>
-    <hyperlink ref="O78" r:id="rId75"/>
-    <hyperlink ref="O79" r:id="rId76"/>
-    <hyperlink ref="O81" r:id="rId77"/>
+    <hyperlink ref="O17" r:id="rId5"/>
+    <hyperlink ref="O19" r:id="rId6"/>
+    <hyperlink ref="O22" r:id="rId7"/>
+    <hyperlink ref="O21" r:id="rId8"/>
+    <hyperlink ref="O23" r:id="rId9"/>
+    <hyperlink ref="O24" r:id="rId10"/>
+    <hyperlink ref="O25" r:id="rId11"/>
+    <hyperlink ref="O28" r:id="rId12"/>
+    <hyperlink ref="O29" r:id="rId13"/>
+    <hyperlink ref="O30" r:id="rId14"/>
+    <hyperlink ref="O31" r:id="rId15"/>
+    <hyperlink ref="O32" r:id="rId16"/>
+    <hyperlink ref="O33" r:id="rId17"/>
+    <hyperlink ref="O34" r:id="rId18"/>
+    <hyperlink ref="O35" r:id="rId19"/>
+    <hyperlink ref="O36" r:id="rId20"/>
+    <hyperlink ref="O37" r:id="rId21"/>
+    <hyperlink ref="O38" r:id="rId22"/>
+    <hyperlink ref="O40" r:id="rId23"/>
+    <hyperlink ref="O42" r:id="rId24"/>
+    <hyperlink ref="O43" r:id="rId25"/>
+    <hyperlink ref="O44" r:id="rId26"/>
+    <hyperlink ref="O45" r:id="rId27"/>
+    <hyperlink ref="O46" r:id="rId28"/>
+    <hyperlink ref="O47" r:id="rId29"/>
+    <hyperlink ref="O49" r:id="rId30"/>
+    <hyperlink ref="O51" r:id="rId31"/>
+    <hyperlink ref="O52" r:id="rId32"/>
+    <hyperlink ref="O53" r:id="rId33"/>
+    <hyperlink ref="O55" r:id="rId34"/>
+    <hyperlink ref="O56" r:id="rId35"/>
+    <hyperlink ref="O58" r:id="rId36"/>
+    <hyperlink ref="O59" r:id="rId37"/>
+    <hyperlink ref="O60" r:id="rId38"/>
+    <hyperlink ref="O61" r:id="rId39"/>
+    <hyperlink ref="O62" r:id="rId40"/>
+    <hyperlink ref="O63" r:id="rId41"/>
+    <hyperlink ref="O64" r:id="rId42"/>
+    <hyperlink ref="O65" r:id="rId43"/>
+    <hyperlink ref="O67" r:id="rId44"/>
+    <hyperlink ref="O68" r:id="rId45"/>
+    <hyperlink ref="O69" r:id="rId46"/>
+    <hyperlink ref="O70" r:id="rId47"/>
+    <hyperlink ref="O73" r:id="rId48"/>
+    <hyperlink ref="O74" r:id="rId49"/>
+    <hyperlink ref="O75" r:id="rId50"/>
+    <hyperlink ref="O76" r:id="rId51"/>
+    <hyperlink ref="O77" r:id="rId52"/>
+    <hyperlink ref="O80" r:id="rId53"/>
+    <hyperlink ref="O82" r:id="rId54"/>
+    <hyperlink ref="O83" r:id="rId55"/>
+    <hyperlink ref="O84" r:id="rId56"/>
+    <hyperlink ref="O85" r:id="rId57"/>
+    <hyperlink ref="O86" r:id="rId58"/>
+    <hyperlink ref="O87" r:id="rId59"/>
+    <hyperlink ref="O88" r:id="rId60"/>
+    <hyperlink ref="O89" r:id="rId61"/>
+    <hyperlink ref="O72" r:id="rId62"/>
+    <hyperlink ref="O20" r:id="rId63"/>
+    <hyperlink ref="O26" r:id="rId64"/>
+    <hyperlink ref="O27" r:id="rId65"/>
+    <hyperlink ref="O50" r:id="rId66"/>
+    <hyperlink ref="O54" r:id="rId67"/>
+    <hyperlink ref="O57" r:id="rId68"/>
+    <hyperlink ref="O66" r:id="rId69"/>
+    <hyperlink ref="O78" r:id="rId70"/>
+    <hyperlink ref="O79" r:id="rId71"/>
+    <hyperlink ref="O81" r:id="rId72"/>
+    <hyperlink ref="O15" r:id="rId73"/>
+    <hyperlink ref="O16" r:id="rId74"/>
+    <hyperlink ref="O18" r:id="rId75"/>
+    <hyperlink ref="O39" r:id="rId76"/>
+    <hyperlink ref="O41" r:id="rId77"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId78"/>

</xml_diff>